<commit_message>
Initiated display ext. services script
</commit_message>
<xml_diff>
--- a/data/subcontractors.xlsx
+++ b/data/subcontractors.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\cbolanos\Desktop\projects\cps-tool\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ACFAA458-8790-4F58-B05B-7199FDA56784}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A0023829-23F9-4C07-A788-EE3F6AB4BDA8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="7050" yWindow="1890" windowWidth="19485" windowHeight="11235" xr2:uid="{7FC67F31-20FD-4FEB-ADE5-67E343098000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{7FC67F31-20FD-4FEB-ADE5-67E343098000}"/>
   </bookViews>
   <sheets>
     <sheet name="Subcontractors" sheetId="1" r:id="rId1"/>
@@ -745,7 +745,7 @@
         <v>1</v>
       </c>
       <c r="E3" s="1">
-        <v>45</v>
+        <v>41.92</v>
       </c>
       <c r="F3" s="1" t="s">
         <v>29</v>

</xml_diff>

<commit_message>
Updated template and subcontractor data
</commit_message>
<xml_diff>
--- a/data/subcontractors.xlsx
+++ b/data/subcontractors.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\cbolanos\Desktop\projects\cps-tool\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{72FF7145-FAC9-4B3E-94CB-FC3EBC6CCC82}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5CA0A4E7-F300-40C8-BAC4-FE6D1809E40F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{7FC67F31-20FD-4FEB-ADE5-67E343098000}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="80" uniqueCount="45">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="83" uniqueCount="46">
   <si>
     <t>name</t>
   </si>
@@ -175,6 +175,9 @@
   </si>
   <si>
     <t>name_long</t>
+  </si>
+  <si>
+    <t>Space rental</t>
   </si>
 </sst>
 </file>
@@ -676,7 +679,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{99868D97-6DB9-4B7B-AE4B-68BC5BA5F035}">
-  <dimension ref="A1:F17"/>
+  <dimension ref="A1:F18"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="2" width="9.140625" style="1"/>
@@ -967,19 +970,19 @@
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A15" s="1" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="B15" s="1" t="s">
         <v>13</v>
       </c>
       <c r="C15" t="s">
-        <v>38</v>
+        <v>45</v>
       </c>
       <c r="D15">
         <v>1</v>
       </c>
       <c r="E15" s="1">
-        <v>670.07</v>
+        <v>0.123</v>
       </c>
       <c r="F15" s="1" t="b">
         <v>0</v>
@@ -987,22 +990,22 @@
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A16" s="1" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>19</v>
+        <v>13</v>
       </c>
       <c r="C16" t="s">
-        <v>3</v>
+        <v>38</v>
       </c>
       <c r="D16">
         <v>1</v>
       </c>
       <c r="E16" s="1">
-        <v>0</v>
+        <v>670.07</v>
       </c>
       <c r="F16" s="1" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.25">
@@ -1013,19 +1016,40 @@
         <v>19</v>
       </c>
       <c r="C17" t="s">
+        <v>3</v>
+      </c>
+      <c r="D17">
+        <v>1</v>
+      </c>
+      <c r="E17" s="1">
+        <v>0</v>
+      </c>
+      <c r="F17" s="1" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A18" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="B18" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="C18" t="s">
         <v>39</v>
       </c>
-      <c r="D17">
-        <v>0</v>
-      </c>
-      <c r="E17" s="1">
+      <c r="D18">
+        <v>0</v>
+      </c>
+      <c r="E18" s="1">
         <v>105</v>
       </c>
-      <c r="F17" s="1" t="b">
+      <c r="F18" s="1" t="b">
         <v>1</v>
       </c>
     </row>
   </sheetData>
+  <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Updated prices for ICO
</commit_message>
<xml_diff>
--- a/data/subcontractors.xlsx
+++ b/data/subcontractors.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\cbolanos\Desktop\projects\cps-tool\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4B95AF45-0836-425E-9CC1-B4FFE8FF5F42}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5FDC20AA-EB0F-4356-8BAD-BC05623C01CB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{7FC67F31-20FD-4FEB-ADE5-67E343098000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{7FC67F31-20FD-4FEB-ADE5-67E343098000}"/>
   </bookViews>
   <sheets>
     <sheet name="Subcontractors" sheetId="1" r:id="rId1"/>
@@ -902,7 +902,7 @@
         <v>2</v>
       </c>
       <c r="E11" s="1">
-        <v>11.5</v>
+        <v>11.75</v>
       </c>
       <c r="F11" s="1" t="b">
         <v>1</v>
@@ -922,7 +922,7 @@
         <v>1</v>
       </c>
       <c r="E12" s="1">
-        <v>12.5</v>
+        <v>12.75</v>
       </c>
       <c r="F12" s="1" t="b">
         <v>1</v>
@@ -942,7 +942,7 @@
         <v>1</v>
       </c>
       <c r="E13" s="1">
-        <v>3.13</v>
+        <v>3.2</v>
       </c>
       <c r="F13" s="1" t="b">
         <v>1</v>
@@ -962,7 +962,7 @@
         <v>1</v>
       </c>
       <c r="E14" s="1">
-        <v>3.13</v>
+        <v>3.2</v>
       </c>
       <c r="F14" s="1" t="b">
         <v>1</v>

</xml_diff>

<commit_message>
Update to subcontractor rates
</commit_message>
<xml_diff>
--- a/data/subcontractors.xlsx
+++ b/data/subcontractors.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\cbolanos\Desktop\projects\cps-tool\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5FDC20AA-EB0F-4356-8BAD-BC05623C01CB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7163781D-8A86-4851-94B3-DF12F309CF95}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{7FC67F31-20FD-4FEB-ADE5-67E343098000}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="83" uniqueCount="46">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="102" uniqueCount="53">
   <si>
     <t>name</t>
   </si>
@@ -178,6 +178,27 @@
   </si>
   <si>
     <t>Space rental</t>
+  </si>
+  <si>
+    <t>12V charge</t>
+  </si>
+  <si>
+    <t>VPC move</t>
+  </si>
+  <si>
+    <t>2-Layer Cargo Bed Coating</t>
+  </si>
+  <si>
+    <t>Protective Coating - Chassis</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Advanced Photoshoot </t>
+  </si>
+  <si>
+    <t>Hourly rate</t>
+  </si>
+  <si>
+    <t>Video shoot</t>
   </si>
 </sst>
 </file>
@@ -219,13 +240,16 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -679,7 +703,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{99868D97-6DB9-4B7B-AE4B-68BC5BA5F035}">
-  <dimension ref="A1:F18"/>
+  <dimension ref="A1:I24"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="2" width="9.140625" style="1"/>
@@ -688,7 +712,7 @@
     <col min="5" max="5" width="9.140625" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>14</v>
       </c>
@@ -708,7 +732,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>15</v>
       </c>
@@ -728,7 +752,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
         <v>15</v>
       </c>
@@ -747,8 +771,11 @@
       <c r="F3" s="1" t="b">
         <v>0</v>
       </c>
-    </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="I3" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
         <v>15</v>
       </c>
@@ -767,8 +794,11 @@
       <c r="F4" s="1" t="b">
         <v>0</v>
       </c>
-    </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="I4">
+        <v>63.75</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
         <v>15</v>
       </c>
@@ -788,7 +818,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
         <v>16</v>
       </c>
@@ -808,7 +838,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
         <v>16</v>
       </c>
@@ -828,7 +858,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
         <v>16</v>
       </c>
@@ -848,7 +878,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A9" s="1" t="s">
         <v>16</v>
       </c>
@@ -868,7 +898,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A10" s="1" t="s">
         <v>16</v>
       </c>
@@ -888,7 +918,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A11" s="1" t="s">
         <v>17</v>
       </c>
@@ -908,7 +938,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A12" s="1" t="s">
         <v>17</v>
       </c>
@@ -916,19 +946,19 @@
         <v>13</v>
       </c>
       <c r="C12" t="s">
-        <v>30</v>
+        <v>47</v>
       </c>
       <c r="D12">
         <v>1</v>
       </c>
       <c r="E12" s="1">
-        <v>12.75</v>
+        <v>6.5</v>
       </c>
       <c r="F12" s="1" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A13" s="1" t="s">
         <v>17</v>
       </c>
@@ -936,19 +966,19 @@
         <v>13</v>
       </c>
       <c r="C13" t="s">
-        <v>37</v>
+        <v>46</v>
       </c>
       <c r="D13">
         <v>1</v>
       </c>
       <c r="E13" s="1">
-        <v>3.2</v>
+        <v>9.19</v>
       </c>
       <c r="F13" s="1" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A14" s="1" t="s">
         <v>17</v>
       </c>
@@ -956,39 +986,41 @@
         <v>13</v>
       </c>
       <c r="C14" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="D14">
         <v>1</v>
       </c>
       <c r="E14" s="1">
-        <v>3.2</v>
+        <f>I4*0.2</f>
+        <v>12.75</v>
       </c>
       <c r="F14" s="1" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A15" s="1" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B15" s="1" t="s">
         <v>13</v>
       </c>
       <c r="C15" t="s">
-        <v>45</v>
+        <v>50</v>
       </c>
       <c r="D15">
         <v>1</v>
       </c>
-      <c r="E15" s="1">
-        <v>15.3</v>
+      <c r="E15" s="3">
+        <f>I4*0.4411</f>
+        <v>28.120124999999998</v>
       </c>
       <c r="F15" s="1" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A16" s="1" t="s">
         <v>17</v>
       </c>
@@ -996,33 +1028,34 @@
         <v>13</v>
       </c>
       <c r="C16" t="s">
-        <v>38</v>
+        <v>52</v>
       </c>
       <c r="D16">
         <v>1</v>
       </c>
-      <c r="E16" s="1">
-        <v>670.07</v>
+      <c r="E16" s="3">
+        <f>I4*0.4902</f>
+        <v>31.250250000000001</v>
       </c>
       <c r="F16" s="1" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A17" s="1" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B17" s="1" t="s">
-        <v>19</v>
+        <v>13</v>
       </c>
       <c r="C17" t="s">
-        <v>3</v>
+        <v>37</v>
       </c>
       <c r="D17">
         <v>1</v>
       </c>
       <c r="E17" s="1">
-        <v>0</v>
+        <v>3.2</v>
       </c>
       <c r="F17" s="1" t="b">
         <v>1</v>
@@ -1030,21 +1063,141 @@
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A18" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="B18" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="C18" t="s">
+        <v>29</v>
+      </c>
+      <c r="D18">
+        <v>1</v>
+      </c>
+      <c r="E18" s="1">
+        <v>3.2</v>
+      </c>
+      <c r="F18" s="1" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A19" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="B19" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="C19" t="s">
+        <v>45</v>
+      </c>
+      <c r="D19">
+        <v>1</v>
+      </c>
+      <c r="E19" s="1">
+        <v>15.3</v>
+      </c>
+      <c r="F19" s="1" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A20" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="B20" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="C20" t="s">
+        <v>48</v>
+      </c>
+      <c r="D20">
+        <v>1</v>
+      </c>
+      <c r="E20" s="1">
+        <v>475.12</v>
+      </c>
+      <c r="F20" s="1" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A21" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="B21" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="C21" t="s">
+        <v>38</v>
+      </c>
+      <c r="D21">
+        <v>1</v>
+      </c>
+      <c r="E21" s="1">
+        <v>670.07</v>
+      </c>
+      <c r="F21" s="1" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="22" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A22" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="B22" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="C22" t="s">
+        <v>49</v>
+      </c>
+      <c r="D22">
+        <v>1</v>
+      </c>
+      <c r="E22" s="1">
+        <v>325</v>
+      </c>
+      <c r="F22" s="1" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A23" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="B18" s="1" t="s">
+      <c r="B23" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="C18" t="s">
+      <c r="C23" t="s">
+        <v>3</v>
+      </c>
+      <c r="D23">
+        <v>1</v>
+      </c>
+      <c r="E23" s="1">
+        <v>0</v>
+      </c>
+      <c r="F23" s="1" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="24" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A24" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="B24" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="C24" t="s">
         <v>39</v>
       </c>
-      <c r="D18">
-        <v>0</v>
-      </c>
-      <c r="E18" s="1">
+      <c r="D24">
+        <v>0</v>
+      </c>
+      <c r="E24" s="1">
         <v>105</v>
       </c>
-      <c r="F18" s="1" t="b">
+      <c r="F24" s="1" t="b">
         <v>1</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Update to subcontractor rates 2
</commit_message>
<xml_diff>
--- a/data/subcontractors.xlsx
+++ b/data/subcontractors.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\cbolanos\Desktop\projects\cps-tool\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7163781D-8A86-4851-94B3-DF12F309CF95}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{40B1D357-FE17-43C1-B4E6-A98009744509}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{7FC67F31-20FD-4FEB-ADE5-67E343098000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{7FC67F31-20FD-4FEB-ADE5-67E343098000}"/>
   </bookViews>
   <sheets>
     <sheet name="Subcontractors" sheetId="1" r:id="rId1"/>
@@ -1038,7 +1038,7 @@
         <v>31.250250000000001</v>
       </c>
       <c r="F16" s="1" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
Changed totals calculation and fixed photoshoot issue
</commit_message>
<xml_diff>
--- a/data/subcontractors.xlsx
+++ b/data/subcontractors.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\cbolanos\Desktop\projects\cps-tool\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{40B1D357-FE17-43C1-B4E6-A98009744509}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C9632294-0503-40D6-8587-C2938441E3B7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{7FC67F31-20FD-4FEB-ADE5-67E343098000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{7FC67F31-20FD-4FEB-ADE5-67E343098000}"/>
   </bookViews>
   <sheets>
     <sheet name="Subcontractors" sheetId="1" r:id="rId1"/>
@@ -763,7 +763,7 @@
         <v>37</v>
       </c>
       <c r="D3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E3" s="1">
         <v>41.92</v>
@@ -1052,7 +1052,7 @@
         <v>37</v>
       </c>
       <c r="D17">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E17" s="1">
         <v>3.2</v>

</xml_diff>